<commit_message>
Atualiza relatório e ajusta gestores de colaboradores
- Substitui RelatorioBancoHoras.xls pela versão atualizada
- Adiciona Josenildo Alves, Shayane Oliveira e Maria Fernanda Gomes ao time de Maria Taciane
- Move Hugo Castro Lopes do time de Alberto para o de Carlos Eduardo

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Saldos_por_Gestor_Ajustado.xlsx
+++ b/public/Saldos_por_Gestor_Ajustado.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B81"/>
+  <dimension ref="A1:B84"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -625,7 +625,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Carlos Eduardo Silva De Oliveira</v>
       </c>
       <c r="B29" t="str">
         <v>Hugo Castro Lopes</v>
@@ -1047,9 +1047,33 @@
         <v>Yuri Castro Gomes</v>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>Maria Taciane Pereira Barbosa</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Josenildo Alves da silva Júnior</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>Maria Taciane Pereira Barbosa</v>
+      </c>
+      <c r="B83" t="str">
+        <v>Shayane Oliveira Ferreira</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>Maria Taciane Pereira Barbosa</v>
+      </c>
+      <c r="B84" t="str">
+        <v>Maria Fernanda Gomes Vieira</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B81"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B84"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adiciona Nayara Soares Kimura ao time de Kemilly Rafaelly
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Saldos_por_Gestor_Ajustado.xlsx
+++ b/public/Saldos_por_Gestor_Ajustado.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B84"/>
+  <dimension ref="A1:B85"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1071,9 +1071,17 @@
         <v>Maria Fernanda Gomes Vieira</v>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>Kemilly Rafaelly Souza Silva</v>
+      </c>
+      <c r="B85" t="str">
+        <v>Nayara Soares Kimura</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B84"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B85"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Substitui gestor Michaell Jean Nunes por Tomas Azevedo Santos
Michaell saiu da empresa; Tomas Azevedo Santos assumiu o cargo.
Equipe (Amanda Santos Costa, Maria Nobre Farias De Franca e o proprio
Tomas) agora vinculada a Tomas Azevedo Santos.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Saldos_por_Gestor_Ajustado.xlsx
+++ b/public/Saldos_por_Gestor_Ajustado.xlsx
@@ -417,7 +417,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Michaell Jean Nunes De Carvalho</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
       <c r="B3" t="str">
         <v>Amanda Santos Costa</v>
@@ -849,7 +849,7 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Michaell Jean Nunes De Carvalho</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
       <c r="B57" t="str">
         <v>Maria Nobre Farias De França</v>
@@ -1009,7 +1009,7 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Michaell Jean Nunes De Carvalho</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
       <c r="B77" t="str">
         <v>Tomás Azevedo Santos</v>

</xml_diff>

<commit_message>
Adiciona Caroline Leite e Rayanne Ferreira a equipe da Kemilly
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Saldos_por_Gestor_Ajustado.xlsx
+++ b/public/Saldos_por_Gestor_Ajustado.xlsx
@@ -121,10 +121,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -156,10 +156,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B85"/>
+  <dimension ref="A1:B87"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1079,9 +1079,25 @@
         <v>Nayara Soares Kimura</v>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>Kemilly Rafaelly Souza Silva</v>
+      </c>
+      <c r="B86" t="str">
+        <v>Caroline Leite</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>Kemilly Rafaelly Souza Silva</v>
+      </c>
+      <c r="B87" t="str">
+        <v>Rayanne Ferreira</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B85"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B87"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Reativa Lianda no painel, na equipe da Suzana
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Saldos_por_Gestor_Ajustado.xlsx
+++ b/public/Saldos_por_Gestor_Ajustado.xlsx
@@ -121,10 +121,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -156,10 +156,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B87"/>
+  <dimension ref="A1:B88"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1009,18 +1009,18 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Tomás Azevedo Santos</v>
+        <v>Suzana Martins Tavares</v>
       </c>
       <c r="B77" t="str">
-        <v>Tomás Azevedo Santos</v>
+        <v>Lianda Melinda Santos Calixto</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
       <c r="B78" t="str">
-        <v>Valesca Meirelle Bezerra Vitória</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
     </row>
     <row r="79">
@@ -1028,31 +1028,31 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B79" t="str">
-        <v>Yasmim Da Rocha Bezerra Barbosa</v>
+        <v>Valesca Meirelle Bezerra Vitória</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B80" t="str">
-        <v>Yasmin Abilia Ferro da Silva</v>
+        <v>Yasmim Da Rocha Bezerra Barbosa</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B81" t="str">
-        <v>Yuri Castro Gomes</v>
+        <v>Yasmin Abilia Ferro da Silva</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B82" t="str">
-        <v>Josenildo Alves da silva Júnior</v>
+        <v>Yuri Castro Gomes</v>
       </c>
     </row>
     <row r="83">
@@ -1060,7 +1060,7 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B83" t="str">
-        <v>Shayane Oliveira Ferreira</v>
+        <v>Josenildo Alves da silva Júnior</v>
       </c>
     </row>
     <row r="84">
@@ -1068,15 +1068,15 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B84" t="str">
-        <v>Maria Fernanda Gomes Vieira</v>
+        <v>Shayane Oliveira Ferreira</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B85" t="str">
-        <v>Nayara Soares Kimura</v>
+        <v>Maria Fernanda Gomes Vieira</v>
       </c>
     </row>
     <row r="86">
@@ -1084,7 +1084,7 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B86" t="str">
-        <v>Caroline Leite</v>
+        <v>Nayara Soares Kimura</v>
       </c>
     </row>
     <row r="87">
@@ -1092,12 +1092,20 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B87" t="str">
+        <v>Caroline Leite</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>Kemilly Rafaelly Souza Silva</v>
+      </c>
+      <c r="B88" t="str">
         <v>Rayanne Ferreira</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B87"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B88"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Move Rodrigo e Sandra para a equipe do Erick Cafe
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Saldos_por_Gestor_Ajustado.xlsx
+++ b/public/Saldos_por_Gestor_Ajustado.xlsx
@@ -937,26 +937,26 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Sem Gestor</v>
       </c>
       <c r="B68" t="str">
-        <v>Rodrigo Augusto Teixeira Dos Santos</v>
+        <v>Romulo Jose Santos Lisboa</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Sem Gestor</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B69" t="str">
-        <v>Romulo Jose Santos Lisboa</v>
+        <v>Rosilene Martins Da Silva</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B70" t="str">
-        <v>Rosilene Martins Da Silva</v>
+        <v>Sabrina Domingos Santos</v>
       </c>
     </row>
     <row r="71">
@@ -964,12 +964,12 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B71" t="str">
-        <v>Sabrina Domingos Santos</v>
+        <v>Rodrigo Augusto Teixeira Dos Santos</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B72" t="str">
         <v>Sandra da Conceição Freitas</v>

</xml_diff>

<commit_message>
Cadastra 17 novos colaboradores em suas equipes
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Saldos_por_Gestor_Ajustado.xlsx
+++ b/public/Saldos_por_Gestor_Ajustado.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B88"/>
+  <dimension ref="A1:B105"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1103,9 +1103,145 @@
         <v>Rayanne Ferreira</v>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>Kemilly Rafaelly Souza Silva</v>
+      </c>
+      <c r="B89" t="str">
+        <v>Luciene Tayná Félix da Silva</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>Kemilly Rafaelly Souza Silva</v>
+      </c>
+      <c r="B90" t="str">
+        <v>Bruna Soares Siqueira</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>Kemilly Rafaelly Souza Silva</v>
+      </c>
+      <c r="B91" t="str">
+        <v>Edlane Silva de Lima</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>Maria Taciane Pereira Barbosa</v>
+      </c>
+      <c r="B92" t="str">
+        <v>Jayane da Silva Dias</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>Maria Taciane Pereira Barbosa</v>
+      </c>
+      <c r="B93" t="str">
+        <v>Rayanne Maria dos Santos Moca</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>Maria Taciane Pereira Barbosa</v>
+      </c>
+      <c r="B94" t="str">
+        <v>Evellyn Vitória Nunes Santos</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>Alberto Luiz Marinho Batista</v>
+      </c>
+      <c r="B95" t="str">
+        <v>Samuel Monteiro da Silva</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>Jonathan Henrique da Conceição Silva</v>
+      </c>
+      <c r="B96" t="str">
+        <v>Juliana Francine Marques da Silva</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>Mariane Santos Sousa</v>
+      </c>
+      <c r="B97" t="str">
+        <v>Juliene Reis Ferreira</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>Ana Clara de Matos Chagas</v>
+      </c>
+      <c r="B98" t="str">
+        <v>Tayna Monaisa Vasconcelos santos</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>Ana Clara de Matos Chagas</v>
+      </c>
+      <c r="B99" t="str">
+        <v>Amanda de Araújo Santos</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>Ana Clara de Matos Chagas</v>
+      </c>
+      <c r="B100" t="str">
+        <v>Auda da Conceição Santos</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>Tomás Azevedo Santos</v>
+      </c>
+      <c r="B101" t="str">
+        <v>Sione Barbosa da Silva</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>Suzana Martins Tavares</v>
+      </c>
+      <c r="B102" t="str">
+        <v>Sabrina Barbosa Machado Mariano</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>Suzana Martins Tavares</v>
+      </c>
+      <c r="B103" t="str">
+        <v>João Paulo Vieira Melo</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>Joao Antonio Tavares Santos</v>
+      </c>
+      <c r="B104" t="str">
+        <v>Crislaine Freire dos Santos</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>Joao Antonio Tavares Santos</v>
+      </c>
+      <c r="B105" t="str">
+        <v>Kledja Nunes da Silva</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B88"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B105"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Move Rayanne Ferreira para Maria Taciane e remove 4 desligados do mapa
Desligados: Kamilla Santos da Silva, Larissa Alexia da Silva Souza, Maria Victoria Souza Araujo Ferro, Thamirys Silvestrini Morales.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Saldos_por_Gestor_Ajustado.xlsx
+++ b/public/Saldos_por_Gestor_Ajustado.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B105"/>
+  <dimension ref="A1:B101"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -705,10 +705,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B39" t="str">
-        <v>Kamilla Santos da Silva</v>
+        <v>Karine Celestino Evangelista dos Santos</v>
       </c>
     </row>
     <row r="40">
@@ -716,7 +716,7 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B40" t="str">
-        <v>Karine Celestino Evangelista dos Santos</v>
+        <v>Kauanne Iwashita Da Silva</v>
       </c>
     </row>
     <row r="41">
@@ -724,63 +724,63 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B41" t="str">
-        <v>Kauanne Iwashita Da Silva</v>
+        <v>Laís Manuelle Santos Pereira</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B42" t="str">
-        <v>Laís Manuelle Santos Pereira</v>
+        <v>Lays da Silva Vieira</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B43" t="str">
-        <v>Larissa Alexia da Silva Souza</v>
+        <v>Leticia Seixas Santos</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Rafaela Alves Mendes</v>
       </c>
       <c r="B44" t="str">
-        <v>Lays da Silva Vieira</v>
+        <v>Letícia Soares Belo</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B45" t="str">
-        <v>Leticia Seixas Santos</v>
+        <v>Luan Santos de Oliveira</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Rafaela Alves Mendes</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B46" t="str">
-        <v>Letícia Soares Belo</v>
+        <v>Luciene Da Silva Nascimento</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B47" t="str">
-        <v>Luan Santos de Oliveira</v>
+        <v>Luciano Torres</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B48" t="str">
-        <v>Luciene Da Silva Nascimento</v>
+        <v>Ludmylla Wolpert Melo</v>
       </c>
     </row>
     <row r="49">
@@ -788,7 +788,7 @@
         <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B49" t="str">
-        <v>Luciano Torres</v>
+        <v>Luiz Fellipe Guedes Santos Silva</v>
       </c>
     </row>
     <row r="50">
@@ -796,111 +796,111 @@
         <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B50" t="str">
-        <v>Ludmylla Wolpert Melo</v>
+        <v>Marcio Alif Santos Silva</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Leidiane Souza</v>
       </c>
       <c r="B51" t="str">
-        <v>Luiz Fellipe Guedes Santos Silva</v>
+        <v>Mariane Santos Sousa</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B52" t="str">
-        <v>Marcio Alif Santos Silva</v>
+        <v>Marília Alice dos Santos Silva</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Leidiane Souza</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B53" t="str">
-        <v>Mariane Santos Sousa</v>
+        <v>Maria Cicília Brito Veiga</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B54" t="str">
-        <v>Marília Alice dos Santos Silva</v>
+        <v>Maria Jeane da Silva Santos</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
       <c r="B55" t="str">
-        <v>Maria Cicília Brito Veiga</v>
+        <v>Maria Nobre Farias De França</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B56" t="str">
-        <v>Maria Jeane da Silva Santos</v>
+        <v>Maria Tatiane Oliveira Santos</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Tomás Azevedo Santos</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B57" t="str">
-        <v>Maria Nobre Farias De França</v>
+        <v>Maryanna Francielly Trajano da Silva</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Joao Antonio Tavares Santos</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B58" t="str">
-        <v>Maria Tatiane Oliveira Santos</v>
+        <v>Natali de Souza Gonzaga</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B59" t="str">
-        <v>Maria Victoria Souza Araujo Ferro</v>
+        <v>Nathalia Vieira Lima</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B60" t="str">
-        <v>Maryanna Francielly Trajano da Silva</v>
+        <v>Paulo Cesar Da Silva Santos Junior</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B61" t="str">
-        <v>Natali de Souza Gonzaga</v>
+        <v>Pedro Lucas Rocha da Fonseca</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B62" t="str">
-        <v>Nathalia Vieira Lima</v>
+        <v>Raquele Fragoso Da Silva</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Suzana Martins Tavares</v>
       </c>
       <c r="B63" t="str">
-        <v>Paulo Cesar Da Silva Santos Junior</v>
+        <v>Ravy Thiago Vieira Da Silva</v>
       </c>
     </row>
     <row r="64">
@@ -908,159 +908,159 @@
         <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B64" t="str">
-        <v>Pedro Lucas Rocha da Fonseca</v>
+        <v>Robéria Gilo Da Silva</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Sem Gestor</v>
       </c>
       <c r="B65" t="str">
-        <v>Raquele Fragoso Da Silva</v>
+        <v>Romulo Jose Santos Lisboa</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Suzana Martins Tavares</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B66" t="str">
-        <v>Ravy Thiago Vieira Da Silva</v>
+        <v>Rosilene Martins Da Silva</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B67" t="str">
-        <v>Robéria Gilo Da Silva</v>
+        <v>Sabrina Domingos Santos</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Sem Gestor</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B68" t="str">
-        <v>Romulo Jose Santos Lisboa</v>
+        <v>Rodrigo Augusto Teixeira Dos Santos</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B69" t="str">
-        <v>Rosilene Martins Da Silva</v>
+        <v>Sandra da Conceição Freitas</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B70" t="str">
-        <v>Sabrina Domingos Santos</v>
+        <v>Thalys Gomes Dos Santos</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B71" t="str">
-        <v>Rodrigo Augusto Teixeira Dos Santos</v>
+        <v>Thamires Emanuelle da Silva</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Suzana Martins Tavares</v>
       </c>
       <c r="B72" t="str">
-        <v>Sandra da Conceição Freitas</v>
+        <v>Thayane Mayara dos Santos</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Suzana Martins Tavares</v>
       </c>
       <c r="B73" t="str">
-        <v>Thalys Gomes Dos Santos</v>
+        <v>Lianda Melinda Santos Calixto</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
       <c r="B74" t="str">
-        <v>Thamires Emanuelle da Silva</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B75" t="str">
-        <v>THAMIRYS SILVESTRINI MORALES</v>
+        <v>Valesca Meirelle Bezerra Vitória</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Suzana Martins Tavares</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B76" t="str">
-        <v>Thayane Mayara dos Santos</v>
+        <v>Yasmim Da Rocha Bezerra Barbosa</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Suzana Martins Tavares</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B77" t="str">
-        <v>Lianda Melinda Santos Calixto</v>
+        <v>Yasmin Abilia Ferro da Silva</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>Tomás Azevedo Santos</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B78" t="str">
-        <v>Tomás Azevedo Santos</v>
+        <v>Yuri Castro Gomes</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B79" t="str">
-        <v>Valesca Meirelle Bezerra Vitória</v>
+        <v>Josenildo Alves da silva Júnior</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B80" t="str">
-        <v>Yasmim Da Rocha Bezerra Barbosa</v>
+        <v>Shayane Oliveira Ferreira</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B81" t="str">
-        <v>Yasmin Abilia Ferro da Silva</v>
+        <v>Maria Fernanda Gomes Vieira</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B82" t="str">
-        <v>Yuri Castro Gomes</v>
+        <v>Nayara Soares Kimura</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B83" t="str">
-        <v>Josenildo Alves da silva Júnior</v>
+        <v>Caroline leite dos santos</v>
       </c>
     </row>
     <row r="84">
@@ -1068,15 +1068,15 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B84" t="str">
-        <v>Shayane Oliveira Ferreira</v>
+        <v>Rayanne Ferreira</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B85" t="str">
-        <v>Maria Fernanda Gomes Vieira</v>
+        <v>Luciene Tayná Félix da Silva</v>
       </c>
     </row>
     <row r="86">
@@ -1084,7 +1084,7 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B86" t="str">
-        <v>Nayara Soares Kimura</v>
+        <v>Bruna Soares Siqueira</v>
       </c>
     </row>
     <row r="87">
@@ -1092,156 +1092,124 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B87" t="str">
-        <v>Caroline leite dos santos</v>
+        <v>Edlane Silva de Lima</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B88" t="str">
-        <v>Rayanne Ferreira</v>
+        <v>Jayane da Silva Dias</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B89" t="str">
-        <v>Luciene Tayná Félix da Silva</v>
+        <v>Rayanne Maria dos Santos Moca</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B90" t="str">
-        <v>Bruna Soares Siqueira</v>
+        <v>Evellyn Vitória Nunes Santos</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B91" t="str">
-        <v>Edlane Silva de Lima</v>
+        <v>Samuel Monteiro da Silva</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B92" t="str">
-        <v>Jayane da Silva Dias</v>
+        <v>Juliana Francine Marques da Silva</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Mariane Santos Sousa</v>
       </c>
       <c r="B93" t="str">
-        <v>Rayanne Maria dos Santos Moca</v>
+        <v>Juliene Reis Ferreira</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B94" t="str">
-        <v>Evellyn Vitória Nunes Santos</v>
+        <v>Tayna Monaisa Vasconcelos santos</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B95" t="str">
-        <v>Samuel Monteiro da Silva</v>
+        <v>Amanda de Araújo Santos</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B96" t="str">
-        <v>Juliana Francine Marques da Silva</v>
+        <v>Auda da Conceição Santos</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>Mariane Santos Sousa</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
       <c r="B97" t="str">
-        <v>Juliene Reis Ferreira</v>
+        <v>Sione Barbosa da Silva</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Suzana Martins Tavares</v>
       </c>
       <c r="B98" t="str">
-        <v>Tayna Monaisa Vasconcelos santos</v>
+        <v>Sabrina Barbosa Machado Mariano</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Suzana Martins Tavares</v>
       </c>
       <c r="B99" t="str">
-        <v>Amanda de Araújo Santos</v>
+        <v>João Paulo Vieira Melo</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B100" t="str">
-        <v>Auda da Conceição Santos</v>
+        <v>Crislaine Freire dos Santos</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>Tomás Azevedo Santos</v>
+        <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B101" t="str">
-        <v>Sione Barbosa da Silva</v>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="str">
-        <v>Suzana Martins Tavares</v>
-      </c>
-      <c r="B102" t="str">
-        <v>Sabrina Barbosa Machado Mariano</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="str">
-        <v>Suzana Martins Tavares</v>
-      </c>
-      <c r="B103" t="str">
-        <v>João Paulo Vieira Melo</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="str">
-        <v>Joao Antonio Tavares Santos</v>
-      </c>
-      <c r="B104" t="str">
-        <v>Crislaine Freire dos Santos</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="str">
-        <v>Joao Antonio Tavares Santos</v>
-      </c>
-      <c r="B105" t="str">
         <v>Kledja Nunes da Silva</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B105"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B101"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adiciona Luis Henrique Batista dos Santos a equipe do Tomas
Remove o nome da lista de excluidos em excel.ts e cadastra a linha
Tomas Azevedo Santos | Luis Henrique Batista dos Santos no mapa de
gestores. Saldo passa a aparecer no painel: +13h57min.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Saldos_por_Gestor_Ajustado.xlsx
+++ b/public/Saldos_por_Gestor_Ajustado.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B101"/>
+  <dimension ref="A1:B102"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1207,9 +1207,17 @@
         <v>Kledja Nunes da Silva</v>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>Tomás Azevedo Santos</v>
+      </c>
+      <c r="B102" t="str">
+        <v>Luís Henrique Batista dos Santos</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B101"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B102"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza horas dos times de Kemilly, Taciane, Suzana e Alberto
Merge de 44 colaboradores a partir dos exports de 01/07 a 02/08.
Yuri Castro (Alberto) e Brunna Isabelly (Ana Clara) nao vieram nos
exports e seguem em 26/07.

Mapa de gestores: Anny Karoline passa da equipe da Mariane para a da
Maria Taciane, e Lianda Melinda sai do mapa. Lianda tambem entra em
EXCLUDED_NAMES para deixar de aparecer no painel -- so tirar do mapa
a deixaria visivel como "Sem Gestor". As horas dela nao foram
atualizadas, conforme pedido.

Remove a secao de divergencia por falta de ajustes do time do Alberto,
resolvida nesta atualizacao. A key dos avisos passa a incluir o indice
porque a Kemilly agora tem dois avisos e o gestor sozinho colidia.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Saldos_por_Gestor_Ajustado.xlsx
+++ b/public/Saldos_por_Gestor_Ajustado.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B102"/>
+  <dimension ref="A1:B101"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -457,7 +457,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Mariane Santos Sousa</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B8" t="str">
         <v>Anny Karoline Andrade Santos</v>
@@ -977,18 +977,18 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Suzana Martins Tavares</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
       <c r="B73" t="str">
-        <v>Lianda Melinda Santos Calixto</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Tomás Azevedo Santos</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B74" t="str">
-        <v>Tomás Azevedo Santos</v>
+        <v>Valesca Meirelle Bezerra Vitória</v>
       </c>
     </row>
     <row r="75">
@@ -996,31 +996,31 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B75" t="str">
-        <v>Valesca Meirelle Bezerra Vitória</v>
+        <v>Yasmim Da Rocha Bezerra Barbosa</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B76" t="str">
-        <v>Yasmim Da Rocha Bezerra Barbosa</v>
+        <v>Yasmin Abilia Ferro da Silva</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B77" t="str">
-        <v>Yasmin Abilia Ferro da Silva</v>
+        <v>Yuri Castro Gomes</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B78" t="str">
-        <v>Yuri Castro Gomes</v>
+        <v>Josenildo Alves da silva Júnior</v>
       </c>
     </row>
     <row r="79">
@@ -1028,7 +1028,7 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B79" t="str">
-        <v>Josenildo Alves da silva Júnior</v>
+        <v>Shayane Oliveira Ferreira</v>
       </c>
     </row>
     <row r="80">
@@ -1036,15 +1036,15 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B80" t="str">
-        <v>Shayane Oliveira Ferreira</v>
+        <v>Maria Fernanda Gomes Vieira</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B81" t="str">
-        <v>Maria Fernanda Gomes Vieira</v>
+        <v>Nayara Soares Kimura</v>
       </c>
     </row>
     <row r="82">
@@ -1052,23 +1052,23 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B82" t="str">
-        <v>Nayara Soares Kimura</v>
+        <v>Caroline leite dos santos</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B83" t="str">
-        <v>Caroline leite dos santos</v>
+        <v>Rayanne Ferreira</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B84" t="str">
-        <v>Rayanne Ferreira</v>
+        <v>Luciene Tayná Félix da Silva</v>
       </c>
     </row>
     <row r="85">
@@ -1076,7 +1076,7 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B85" t="str">
-        <v>Luciene Tayná Félix da Silva</v>
+        <v>Bruna Soares Siqueira</v>
       </c>
     </row>
     <row r="86">
@@ -1084,15 +1084,15 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B86" t="str">
-        <v>Bruna Soares Siqueira</v>
+        <v>Edlane Silva de Lima</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B87" t="str">
-        <v>Edlane Silva de Lima</v>
+        <v>Jayane da Silva Dias</v>
       </c>
     </row>
     <row r="88">
@@ -1100,7 +1100,7 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B88" t="str">
-        <v>Jayane da Silva Dias</v>
+        <v>Rayanne Maria dos Santos Moca</v>
       </c>
     </row>
     <row r="89">
@@ -1108,39 +1108,39 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B89" t="str">
-        <v>Rayanne Maria dos Santos Moca</v>
+        <v>Evellyn Vitória Nunes Santos</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B90" t="str">
-        <v>Evellyn Vitória Nunes Santos</v>
+        <v>Samuel Monteiro da Silva</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B91" t="str">
-        <v>Samuel Monteiro da Silva</v>
+        <v>Juliana Francine Marques da Silva</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Mariane Santos Sousa</v>
       </c>
       <c r="B92" t="str">
-        <v>Juliana Francine Marques da Silva</v>
+        <v>Juliene Reis Ferreira</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>Mariane Santos Sousa</v>
+        <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B93" t="str">
-        <v>Juliene Reis Ferreira</v>
+        <v>Tayna Monaisa Vasconcelos santos</v>
       </c>
     </row>
     <row r="94">
@@ -1148,7 +1148,7 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B94" t="str">
-        <v>Tayna Monaisa Vasconcelos santos</v>
+        <v>Amanda de Araújo Santos</v>
       </c>
     </row>
     <row r="95">
@@ -1156,23 +1156,23 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B95" t="str">
-        <v>Amanda de Araújo Santos</v>
+        <v>Auda da Conceição Santos</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
       <c r="B96" t="str">
-        <v>Auda da Conceição Santos</v>
+        <v>Sione Barbosa da Silva</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>Tomás Azevedo Santos</v>
+        <v>Suzana Martins Tavares</v>
       </c>
       <c r="B97" t="str">
-        <v>Sione Barbosa da Silva</v>
+        <v>Sabrina Barbosa Machado Mariano</v>
       </c>
     </row>
     <row r="98">
@@ -1180,15 +1180,15 @@
         <v>Suzana Martins Tavares</v>
       </c>
       <c r="B98" t="str">
-        <v>Sabrina Barbosa Machado Mariano</v>
+        <v>João Paulo Vieira Melo</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>Suzana Martins Tavares</v>
+        <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B99" t="str">
-        <v>João Paulo Vieira Melo</v>
+        <v>Crislaine Freire dos Santos</v>
       </c>
     </row>
     <row r="100">
@@ -1196,28 +1196,20 @@
         <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B100" t="str">
-        <v>Crislaine Freire dos Santos</v>
+        <v>Kledja Nunes da Silva</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>Joao Antonio Tavares Santos</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
       <c r="B101" t="str">
-        <v>Kledja Nunes da Silva</v>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="str">
-        <v>Tomás Azevedo Santos</v>
-      </c>
-      <c r="B102" t="str">
         <v>Luís Henrique Batista dos Santos</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B102"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B101"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>